<commit_message>
Correcao do campos horas e adição de xp do curso
</commit_message>
<xml_diff>
--- a/data/acompanhamento/trilhas/Applied Finance in Python.xlsx
+++ b/data/acompanhamento/trilhas/Applied Finance in Python.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,20 +446,25 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>xp_curso</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>ordem_para_assistir</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>tipo_trilha</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>data_final_para_assistir</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>obrigatoriedade_curso</t>
         </is>
@@ -476,19 +481,20 @@
           <t>Introduction to Portfolio Risk Management in Python</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>4 hr</t>
-        </is>
+      <c r="C2" t="n">
+        <v>4</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>4250</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -503,19 +509,20 @@
           <t>Quantitative Risk Management in Python</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>4 hr</t>
-        </is>
+      <c r="C3" t="n">
+        <v>4</v>
       </c>
       <c r="D3" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -530,19 +537,20 @@
           <t>Credit Risk Modeling in Python</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>4 hr</t>
-        </is>
+      <c r="C4" t="n">
+        <v>4</v>
       </c>
       <c r="D4" t="n">
+        <v>4850</v>
+      </c>
+      <c r="E4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="n">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -557,19 +565,20 @@
           <t>GARCH Models in Python</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>4 hr</t>
-        </is>
+      <c r="C5" t="n">
+        <v>4</v>
       </c>
       <c r="D5" t="n">
+        <v>3950</v>
+      </c>
+      <c r="E5" t="n">
         <v>3</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>